<commit_message>
Fix school quota recommendation: restrict 实验学校 and 上师附中 to Pudong district only
</commit_message>
<xml_diff>
--- a/dataref/2025上海高中学校排名名单.xlsx
+++ b/dataref/2025上海高中学校排名名单.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\high-school-apply\dataref\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B106D87-BE51-44BA-B55F-982A723E35DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A3B5D4C-2590-4536-A8F1-0116B549C64B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6384" yWindow="936" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{20660486-D41A-4902-9432-A4CC4F9D5694}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{20660486-D41A-4902-9432-A4CC4F9D5694}"/>
   </bookViews>
   <sheets>
     <sheet name="汇总" sheetId="2" r:id="rId1"/>
@@ -6607,6 +6607,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{787A588E-310A-4D54-83BE-89CA5695AF2B}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M284"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6666,7 +6667,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -6707,7 +6708,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -6745,7 +6746,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
@@ -6786,7 +6787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -6827,7 +6828,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -6868,7 +6869,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>23</v>
       </c>
@@ -6909,7 +6910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>25</v>
       </c>
@@ -6950,7 +6951,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -6991,7 +6992,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>30</v>
       </c>
@@ -7032,7 +7033,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
@@ -7073,7 +7074,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
@@ -7114,7 +7115,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>34</v>
       </c>
@@ -7155,7 +7156,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>36</v>
       </c>
@@ -7196,7 +7197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>37</v>
       </c>
@@ -7278,7 +7279,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>41</v>
       </c>
@@ -7319,7 +7320,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>42</v>
       </c>
@@ -7360,7 +7361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>44</v>
       </c>
@@ -7401,7 +7402,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>46</v>
       </c>
@@ -7442,7 +7443,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>47</v>
       </c>
@@ -7483,7 +7484,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>49</v>
       </c>
@@ -7506,7 +7507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>51</v>
       </c>
@@ -7547,7 +7548,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
@@ -7588,7 +7589,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
@@ -7629,7 +7630,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
@@ -7670,7 +7671,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>57</v>
       </c>
@@ -7711,7 +7712,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>58</v>
       </c>
@@ -7752,7 +7753,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>60</v>
       </c>
@@ -7793,7 +7794,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>62</v>
       </c>
@@ -7816,7 +7817,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>64</v>
       </c>
@@ -7857,7 +7858,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>65</v>
       </c>
@@ -7898,7 +7899,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>66</v>
       </c>
@@ -7939,7 +7940,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>321</v>
       </c>
@@ -8021,7 +8022,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>68</v>
       </c>
@@ -8050,7 +8051,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>69</v>
       </c>
@@ -8091,7 +8092,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>70</v>
       </c>
@@ -8120,7 +8121,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>71</v>
       </c>
@@ -8161,7 +8162,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>73</v>
       </c>
@@ -8202,7 +8203,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>74</v>
       </c>
@@ -8243,7 +8244,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>75</v>
       </c>
@@ -8281,7 +8282,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>76</v>
       </c>
@@ -8319,7 +8320,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>77</v>
       </c>
@@ -8360,7 +8361,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>78</v>
       </c>
@@ -8401,7 +8402,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>79</v>
       </c>
@@ -8442,7 +8443,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>80</v>
       </c>
@@ -8471,7 +8472,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>82</v>
       </c>
@@ -8506,7 +8507,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>83</v>
       </c>
@@ -8547,7 +8548,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>84</v>
       </c>
@@ -8576,7 +8577,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>86</v>
       </c>
@@ -8617,7 +8618,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>87</v>
       </c>
@@ -8658,7 +8659,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>88</v>
       </c>
@@ -8699,7 +8700,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>324</v>
       </c>
@@ -8728,7 +8729,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>90</v>
       </c>
@@ -8769,7 +8770,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>91</v>
       </c>
@@ -8810,7 +8811,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>93</v>
       </c>
@@ -8851,7 +8852,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>94</v>
       </c>
@@ -8892,7 +8893,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>95</v>
       </c>
@@ -8933,7 +8934,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>96</v>
       </c>
@@ -8974,7 +8975,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>97</v>
       </c>
@@ -9003,7 +9004,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>98</v>
       </c>
@@ -9044,7 +9045,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>99</v>
       </c>
@@ -9085,7 +9086,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>100</v>
       </c>
@@ -9126,7 +9127,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>325</v>
       </c>
@@ -9155,7 +9156,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>101</v>
       </c>
@@ -9196,7 +9197,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>102</v>
       </c>
@@ -9225,7 +9226,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>103</v>
       </c>
@@ -9266,7 +9267,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>104</v>
       </c>
@@ -9295,7 +9296,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>105</v>
       </c>
@@ -9336,7 +9337,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>106</v>
       </c>
@@ -9365,7 +9366,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>107</v>
       </c>
@@ -9394,7 +9395,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>108</v>
       </c>
@@ -9423,7 +9424,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>109</v>
       </c>
@@ -9464,7 +9465,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>110</v>
       </c>
@@ -9505,7 +9506,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>111</v>
       </c>
@@ -9546,7 +9547,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>112</v>
       </c>
@@ -9587,7 +9588,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>113</v>
       </c>
@@ -9616,7 +9617,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>114</v>
       </c>
@@ -9645,7 +9646,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>115</v>
       </c>
@@ -9674,7 +9675,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>116</v>
       </c>
@@ -9703,7 +9704,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>118</v>
       </c>
@@ -9732,7 +9733,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>119</v>
       </c>
@@ -9761,7 +9762,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>120</v>
       </c>
@@ -9802,7 +9803,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>122</v>
       </c>
@@ -9843,7 +9844,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>123</v>
       </c>
@@ -9884,7 +9885,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>124</v>
       </c>
@@ -9925,7 +9926,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>125</v>
       </c>
@@ -9954,7 +9955,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>126</v>
       </c>
@@ -9983,7 +9984,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>127</v>
       </c>
@@ -10012,7 +10013,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>128</v>
       </c>
@@ -10041,7 +10042,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>129</v>
       </c>
@@ -10082,7 +10083,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>130</v>
       </c>
@@ -10111,7 +10112,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>326</v>
       </c>
@@ -10140,7 +10141,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>131</v>
       </c>
@@ -10169,7 +10170,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>132</v>
       </c>
@@ -10198,7 +10199,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>133</v>
       </c>
@@ -10227,7 +10228,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>134</v>
       </c>
@@ -10268,7 +10269,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>135</v>
       </c>
@@ -10297,7 +10298,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>136</v>
       </c>
@@ -10326,7 +10327,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>137</v>
       </c>
@@ -10355,7 +10356,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>138</v>
       </c>
@@ -10384,7 +10385,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>139</v>
       </c>
@@ -10416,7 +10417,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>140</v>
       </c>
@@ -10457,7 +10458,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>141</v>
       </c>
@@ -10486,7 +10487,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>142</v>
       </c>
@@ -10509,7 +10510,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>143</v>
       </c>
@@ -10550,7 +10551,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>144</v>
       </c>
@@ -10579,7 +10580,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>145</v>
       </c>
@@ -10608,7 +10609,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>146</v>
       </c>
@@ -10649,7 +10650,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>147</v>
       </c>
@@ -10678,7 +10679,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>148</v>
       </c>
@@ -10707,7 +10708,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>149</v>
       </c>
@@ -10730,7 +10731,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>150</v>
       </c>
@@ -10759,7 +10760,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>151</v>
       </c>
@@ -10788,7 +10789,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>152</v>
       </c>
@@ -10817,7 +10818,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>153</v>
       </c>
@@ -10846,7 +10847,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>154</v>
       </c>
@@ -10875,7 +10876,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>155</v>
       </c>
@@ -10904,7 +10905,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>156</v>
       </c>
@@ -10933,7 +10934,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>157</v>
       </c>
@@ -10962,7 +10963,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>158</v>
       </c>
@@ -10991,7 +10992,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>159</v>
       </c>
@@ -11014,7 +11015,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>160</v>
       </c>
@@ -11043,7 +11044,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>161</v>
       </c>
@@ -11084,7 +11085,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>162</v>
       </c>
@@ -11113,7 +11114,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>163</v>
       </c>
@@ -11142,7 +11143,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>164</v>
       </c>
@@ -11171,7 +11172,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>165</v>
       </c>
@@ -11200,7 +11201,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>166</v>
       </c>
@@ -11229,7 +11230,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>167</v>
       </c>
@@ -11258,7 +11259,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>168</v>
       </c>
@@ -11287,7 +11288,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>169</v>
       </c>
@@ -11316,7 +11317,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>170</v>
       </c>
@@ -11357,7 +11358,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>171</v>
       </c>
@@ -11386,7 +11387,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>172</v>
       </c>
@@ -11415,7 +11416,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>173</v>
       </c>
@@ -11444,7 +11445,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>174</v>
       </c>
@@ -11473,7 +11474,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>175</v>
       </c>
@@ -11502,7 +11503,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>176</v>
       </c>
@@ -11531,7 +11532,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>177</v>
       </c>
@@ -11560,7 +11561,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>178</v>
       </c>
@@ -11589,7 +11590,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>179</v>
       </c>
@@ -11618,7 +11619,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>180</v>
       </c>
@@ -11647,7 +11648,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>181</v>
       </c>
@@ -11676,7 +11677,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>182</v>
       </c>
@@ -11705,7 +11706,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>183</v>
       </c>
@@ -11734,7 +11735,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>184</v>
       </c>
@@ -11775,7 +11776,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>185</v>
       </c>
@@ -11804,7 +11805,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>186</v>
       </c>
@@ -11833,7 +11834,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>187</v>
       </c>
@@ -11862,7 +11863,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>188</v>
       </c>
@@ -11891,7 +11892,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>189</v>
       </c>
@@ -11920,7 +11921,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="6" t="s">
         <v>329</v>
       </c>
@@ -11949,7 +11950,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>190</v>
       </c>
@@ -11978,7 +11979,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="6" t="s">
         <v>332</v>
       </c>
@@ -12007,7 +12008,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>191</v>
       </c>
@@ -12036,7 +12037,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>192</v>
       </c>
@@ -12065,7 +12066,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>193</v>
       </c>
@@ -12094,7 +12095,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>194</v>
       </c>
@@ -12135,7 +12136,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>195</v>
       </c>
@@ -12164,7 +12165,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>196</v>
       </c>
@@ -12193,7 +12194,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>197</v>
       </c>
@@ -12222,7 +12223,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>198</v>
       </c>
@@ -12251,7 +12252,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>199</v>
       </c>
@@ -12280,7 +12281,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>200</v>
       </c>
@@ -12309,7 +12310,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>201</v>
       </c>
@@ -12338,7 +12339,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>202</v>
       </c>
@@ -12367,7 +12368,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>203</v>
       </c>
@@ -12396,7 +12397,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>204</v>
       </c>
@@ -12425,7 +12426,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>205</v>
       </c>
@@ -12454,7 +12455,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>206</v>
       </c>
@@ -12483,7 +12484,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>207</v>
       </c>
@@ -12512,7 +12513,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>208</v>
       </c>
@@ -12541,7 +12542,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>209</v>
       </c>
@@ -12570,7 +12571,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>210</v>
       </c>
@@ -12599,7 +12600,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>211</v>
       </c>
@@ -12628,7 +12629,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>212</v>
       </c>
@@ -12657,7 +12658,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>213</v>
       </c>
@@ -12686,7 +12687,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>214</v>
       </c>
@@ -12715,7 +12716,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>215</v>
       </c>
@@ -12744,7 +12745,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>216</v>
       </c>
@@ -12773,7 +12774,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>217</v>
       </c>
@@ -12802,7 +12803,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>218</v>
       </c>
@@ -12831,7 +12832,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>219</v>
       </c>
@@ -12860,7 +12861,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>220</v>
       </c>
@@ -12889,7 +12890,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>221</v>
       </c>
@@ -12918,7 +12919,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>222</v>
       </c>
@@ -12947,7 +12948,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>223</v>
       </c>
@@ -12976,7 +12977,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>224</v>
       </c>
@@ -13005,7 +13006,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>225</v>
       </c>
@@ -13034,7 +13035,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>226</v>
       </c>
@@ -13063,7 +13064,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>227</v>
       </c>
@@ -13092,7 +13093,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>228</v>
       </c>
@@ -13121,7 +13122,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>229</v>
       </c>
@@ -13150,7 +13151,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>230</v>
       </c>
@@ -13179,7 +13180,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>231</v>
       </c>
@@ -13208,7 +13209,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>232</v>
       </c>
@@ -13237,7 +13238,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>233</v>
       </c>
@@ -13266,7 +13267,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>234</v>
       </c>
@@ -13295,7 +13296,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>235</v>
       </c>
@@ -13324,7 +13325,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>236</v>
       </c>
@@ -13353,7 +13354,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>237</v>
       </c>
@@ -13382,7 +13383,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>238</v>
       </c>
@@ -13411,7 +13412,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>239</v>
       </c>
@@ -13440,7 +13441,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>240</v>
       </c>
@@ -13469,7 +13470,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>241</v>
       </c>
@@ -13498,7 +13499,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>242</v>
       </c>
@@ -13527,7 +13528,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>243</v>
       </c>
@@ -13556,7 +13557,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="210" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>244</v>
       </c>
@@ -13585,7 +13586,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="211" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>245</v>
       </c>
@@ -13614,7 +13615,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="212" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>246</v>
       </c>
@@ -13643,7 +13644,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="213" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>247</v>
       </c>
@@ -13672,7 +13673,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="214" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="6" t="s">
         <v>333</v>
       </c>
@@ -13701,7 +13702,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="215" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>248</v>
       </c>
@@ -13730,7 +13731,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="216" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>249</v>
       </c>
@@ -13759,7 +13760,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>250</v>
       </c>
@@ -13788,7 +13789,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>251</v>
       </c>
@@ -13817,7 +13818,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>252</v>
       </c>
@@ -13846,7 +13847,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>253</v>
       </c>
@@ -13875,7 +13876,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>254</v>
       </c>
@@ -13904,7 +13905,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>255</v>
       </c>
@@ -13933,7 +13934,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>256</v>
       </c>
@@ -13962,7 +13963,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>257</v>
       </c>
@@ -13991,7 +13992,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="225" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>258</v>
       </c>
@@ -14020,7 +14021,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="226" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>259</v>
       </c>
@@ -14049,7 +14050,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="227" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>260</v>
       </c>
@@ -14078,7 +14079,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="228" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>261</v>
       </c>
@@ -14107,7 +14108,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="229" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
         <v>262</v>
       </c>
@@ -14136,7 +14137,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="230" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>263</v>
       </c>
@@ -14165,7 +14166,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="231" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>264</v>
       </c>
@@ -14194,7 +14195,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="232" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
         <v>265</v>
       </c>
@@ -14223,7 +14224,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="233" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>266</v>
       </c>
@@ -14252,7 +14253,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="234" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>267</v>
       </c>
@@ -14281,7 +14282,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="235" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>268</v>
       </c>
@@ -14310,7 +14311,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="236" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
         <v>269</v>
       </c>
@@ -14339,7 +14340,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="237" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>270</v>
       </c>
@@ -14368,7 +14369,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="238" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
         <v>271</v>
       </c>
@@ -14397,7 +14398,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="239" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
         <v>272</v>
       </c>
@@ -14426,7 +14427,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="240" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
         <v>273</v>
       </c>
@@ -14455,7 +14456,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="241" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
         <v>274</v>
       </c>
@@ -14484,7 +14485,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="242" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
         <v>275</v>
       </c>
@@ -14513,7 +14514,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="243" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="2" t="s">
         <v>276</v>
       </c>
@@ -14542,7 +14543,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="244" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
         <v>277</v>
       </c>
@@ -14571,7 +14572,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="245" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
         <v>278</v>
       </c>
@@ -14600,7 +14601,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="246" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
         <v>279</v>
       </c>
@@ -14629,7 +14630,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="247" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="2" t="s">
         <v>280</v>
       </c>
@@ -14658,7 +14659,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="248" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="2" t="s">
         <v>281</v>
       </c>
@@ -14687,7 +14688,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="249" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="2" t="s">
         <v>282</v>
       </c>
@@ -14716,7 +14717,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="250" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="2" t="s">
         <v>283</v>
       </c>
@@ -14745,7 +14746,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="251" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="2" t="s">
         <v>284</v>
       </c>
@@ -14774,7 +14775,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="252" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="6" t="s">
         <v>334</v>
       </c>
@@ -14803,7 +14804,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="253" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="2" t="s">
         <v>285</v>
       </c>
@@ -14832,7 +14833,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="254" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="2" t="s">
         <v>286</v>
       </c>
@@ -14861,7 +14862,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="255" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="2" t="s">
         <v>287</v>
       </c>
@@ -14890,7 +14891,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="256" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="2" t="s">
         <v>288</v>
       </c>
@@ -14919,7 +14920,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="257" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
         <v>289</v>
       </c>
@@ -14948,7 +14949,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="258" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
         <v>290</v>
       </c>
@@ -14977,7 +14978,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="259" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
         <v>291</v>
       </c>
@@ -15000,7 +15001,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="260" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
         <v>292</v>
       </c>
@@ -15029,7 +15030,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="261" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
         <v>293</v>
       </c>
@@ -15058,7 +15059,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="262" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" s="2" t="s">
         <v>294</v>
       </c>
@@ -15087,7 +15088,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="263" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="2" t="s">
         <v>295</v>
       </c>
@@ -15116,7 +15117,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="264" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="2" t="s">
         <v>296</v>
       </c>
@@ -15145,7 +15146,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="265" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="2" t="s">
         <v>297</v>
       </c>
@@ -15174,7 +15175,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="266" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="2" t="s">
         <v>298</v>
       </c>
@@ -15203,7 +15204,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="267" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="2" t="s">
         <v>299</v>
       </c>
@@ -15232,7 +15233,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="268" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="2" t="s">
         <v>300</v>
       </c>
@@ -15261,7 +15262,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="269" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="2" t="s">
         <v>301</v>
       </c>
@@ -15290,7 +15291,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="270" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="2" t="s">
         <v>302</v>
       </c>
@@ -15319,7 +15320,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="271" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="2" t="s">
         <v>303</v>
       </c>
@@ -15342,7 +15343,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="272" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="2" t="s">
         <v>304</v>
       </c>
@@ -15371,7 +15372,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="273" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="2" t="s">
         <v>305</v>
       </c>
@@ -15400,7 +15401,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="274" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="2" t="s">
         <v>306</v>
       </c>
@@ -15429,7 +15430,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="275" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="2" t="s">
         <v>307</v>
       </c>
@@ -15458,7 +15459,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="276" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="2" t="s">
         <v>308</v>
       </c>
@@ -15487,7 +15488,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="277" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="2" t="s">
         <v>309</v>
       </c>
@@ -15516,7 +15517,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="278" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="2" t="s">
         <v>310</v>
       </c>
@@ -15545,7 +15546,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="279" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
         <v>311</v>
       </c>
@@ -15574,7 +15575,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="280" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
         <v>312</v>
       </c>
@@ -15603,7 +15604,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="281" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="2" t="s">
         <v>313</v>
       </c>
@@ -15632,7 +15633,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="282" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="2" t="s">
         <v>314</v>
       </c>
@@ -15661,7 +15662,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="283" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="2" t="s">
         <v>315</v>
       </c>
@@ -15678,7 +15679,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="284" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:13" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
         <v>317</v>
       </c>
@@ -15696,7 +15697,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M284" xr:uid="{787A588E-310A-4D54-83BE-89CA5695AF2B}"/>
+  <autoFilter ref="A1:M284" xr:uid="{787A588E-310A-4D54-83BE-89CA5695AF2B}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="委属市重"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>